<commit_message>
Fix: create upload directories and handle video/webm as audio
</commit_message>
<xml_diff>
--- a/data/applications/applications.xlsx
+++ b/data/applications/applications.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -517,9 +517,68 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Panthadip Maji</v>
+      </c>
+      <c r="B3" t="str">
+        <v>majipanthadip@gmail.com</v>
+      </c>
+      <c r="C3" t="str">
+        <v>1772926457704-754730388.pdf</v>
+      </c>
+      <c r="D3" t="str">
+        <v>1772926476793-470080063.webm</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="G3" t="str">
+        <v>12.97736531081203</v>
+      </c>
+      <c r="H3" t="str">
+        <v>77.66594146593036</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>daint01</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Data Analyst Intern</v>
+      </c>
+      <c r="M3" t="str">
+        <v>2026-03-07T23:34:24.427Z</v>
+      </c>
+      <c r="N3" t="str">
+        <v>1tPsV3IwHx0opL0elQnhBsk1f9A4-UwUg</v>
+      </c>
+      <c r="O3" t="str">
+        <v>https://drive.google.com/file/d/1tPsV3IwHx0opL0elQnhBsk1f9A4-UwUg/view?usp=drivesdk</v>
+      </c>
+      <c r="P3" t="str">
+        <v>1zWAMSLizgpZJGYiMXr5T00IpDH2fssya</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>https://drive.google.com/file/d/1zWAMSLizgpZJGYiMXr5T00IpDH2fssya/view?usp=drivesdk</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>